<commit_message>
upto day day 45 completed
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L93"/>
+  <dimension ref="A1:L92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -934,21 +934,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ATGL</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Adani Total Gas Ltd</t>
+          <t>Axis Bank Ltd</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1.39</v>
+        <v>4.97</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -956,136 +956,140 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>16.8</v>
+        <v>8.23</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>-8.68</v>
+      </c>
+      <c r="I11" t="n">
+        <v>-38.36</v>
+      </c>
       <c r="J11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Axis Bank Ltd</t>
+          <t>Bajaj Auto Ltd</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>4.97</v>
+        <v>0.76</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>8.23</v>
+        <v>0.16</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Asset Light</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>-8.68</v>
+        <v>3.67</v>
       </c>
       <c r="I12" t="n">
-        <v>-38.36</v>
+        <v>74</v>
       </c>
       <c r="J12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K12" t="b">
         <v>0</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bajaj Auto Ltd</t>
+          <t>Bajaj Finserv Ltd</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.76</v>
+        <v>-2.99</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Accrual Risk</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.16</v>
+        <v>9.93</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Asset Light</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>3.67</v>
+        <v>24.34</v>
       </c>
       <c r="I13" t="n">
-        <v>74</v>
+        <v>-194.77</v>
       </c>
       <c r="J13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K13" t="b">
         <v>0</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>BAJAJHLDNG</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Bajaj Finserv Ltd</t>
+          <t>Bajaj Holdings &amp; Investment Ltd</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1094,7 +1098,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>-2.99</v>
+        <v>0.34</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1102,7 +1106,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>9.93</v>
+        <v>27.73</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1110,32 +1114,32 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>24.34</v>
+        <v>7.02</v>
       </c>
       <c r="I14" t="n">
-        <v>-194.77</v>
+        <v>94.05</v>
       </c>
       <c r="J14" t="b">
+        <v>0</v>
+      </c>
+      <c r="K14" t="b">
         <v>1</v>
       </c>
-      <c r="K14" t="b">
-        <v>0</v>
-      </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BAJAJHLDNG</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Bajaj Holdings &amp; Investment Ltd</t>
+          <t>Bajaj Finance Ltd</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1144,7 +1148,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.34</v>
+        <v>-3.76</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1152,7 +1156,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>27.73</v>
+        <v>13.04</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1160,32 +1164,32 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>7.02</v>
+        <v>24.59</v>
       </c>
       <c r="I15" t="n">
-        <v>94.05</v>
+        <v>-496.5</v>
       </c>
       <c r="J15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>BANKBARODA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Bajaj Finance Ltd</t>
+          <t>Bank of Baroda</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1194,26 +1198,26 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>-3.76</v>
+        <v>3.47</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Accrual Risk</t>
+          <t>High Quality</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>13.04</v>
+        <v>1.09</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Asset Light</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>24.59</v>
+        <v>-19.93</v>
       </c>
       <c r="I16" t="n">
-        <v>-496.5</v>
+        <v>-17.03</v>
       </c>
       <c r="J16" t="b">
         <v>1</v>
@@ -1230,21 +1234,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BANKBARODA</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Bank of Baroda</t>
+          <t>Bharat Electronics Ltd</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3.47</v>
+        <v>1.43</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1252,49 +1256,49 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>1.09</v>
+        <v>29.23</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Asset Light</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>-19.93</v>
+        <v>-9.92</v>
       </c>
       <c r="I17" t="n">
-        <v>-17.03</v>
+        <v>-25.04</v>
       </c>
       <c r="J17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K17" t="b">
         <v>0</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Bharat Electronics Ltd</t>
+          <t>Bharti Airtel Ltd</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1.43</v>
+        <v>3.33</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1302,7 +1306,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>29.23</v>
+        <v>34.06</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1310,10 +1314,10 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>-9.92</v>
+        <v>24.79</v>
       </c>
       <c r="I18" t="n">
-        <v>-25.04</v>
+        <v>35.52</v>
       </c>
       <c r="J18" t="b">
         <v>0</v>
@@ -1330,122 +1334,122 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>BHEL</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Bharti Airtel Ltd</t>
+          <t xml:space="preserve">Bharat Heavy Electricals Limited
+</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3.33</v>
+        <v>-2.21</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Accrual Risk</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>34.06</v>
+        <v>5.57</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>24.79</v>
+        <v>23.77</v>
       </c>
       <c r="I19" t="n">
-        <v>35.52</v>
+        <v>-335.02</v>
       </c>
       <c r="J19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K19" t="b">
         <v>0</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Distress Signal</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BHEL</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bharat Heavy Electricals Limited
-</t>
+          <t>Bosch Ltd</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>-2.21</v>
+        <v>1.07</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Accrual Risk</t>
+          <t>High Quality</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>5.57</v>
+        <v>1.69</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Asset Light</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>23.77</v>
+        <v>34.96</v>
       </c>
       <c r="I20" t="n">
-        <v>-335.02</v>
+        <v>73.31999999999999</v>
       </c>
       <c r="J20" t="b">
+        <v>0</v>
+      </c>
+      <c r="K20" t="b">
         <v>1</v>
       </c>
-      <c r="K20" t="b">
-        <v>0</v>
-      </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Distress Signal</t>
+          <t>Liquidating Assets</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>BPCL</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Bosch Ltd</t>
+          <t>Bharat Petroleum Corporation Ltd</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1.07</v>
+        <v>2.49</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1453,7 +1457,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>1.69</v>
+        <v>2.35</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1461,41 +1465,41 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>34.96</v>
+        <v>67.17</v>
       </c>
       <c r="I21" t="n">
-        <v>73.31999999999999</v>
+        <v>57.65</v>
       </c>
       <c r="J21" t="b">
         <v>0</v>
       </c>
       <c r="K21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Liquidating Assets</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Bharat Petroleum Corporation Ltd</t>
+          <t>Britannia Industries Ltd</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>2.49</v>
+        <v>1.05</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1503,7 +1507,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.35</v>
+        <v>2.84</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1511,10 +1515,10 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>67.17</v>
+        <v>193.68</v>
       </c>
       <c r="I22" t="n">
-        <v>57.65</v>
+        <v>96.31</v>
       </c>
       <c r="J22" t="b">
         <v>0</v>
@@ -1524,28 +1528,28 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Liquidating Assets</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>CANBK</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Britannia Industries Ltd</t>
+          <t>Canara Bank</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1.05</v>
+        <v>4.07</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1553,7 +1557,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.84</v>
+        <v>1.58</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1561,10 +1565,10 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>193.68</v>
+        <v>23.4</v>
       </c>
       <c r="I23" t="n">
-        <v>96.31</v>
+        <v>28.81</v>
       </c>
       <c r="J23" t="b">
         <v>0</v>
@@ -1574,19 +1578,19 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Liquidating Assets</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CANBK</t>
+          <t>CHOLAFIN</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Canara Bank</t>
+          <t>Cholamandalam Investment &amp; Finance Company Ltd</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1595,65 +1599,66 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>4.07</v>
+        <v>-6.2</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Accrual Risk</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>1.58</v>
+        <v>14.9</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Asset Light</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>23.4</v>
+        <v>106.27</v>
       </c>
       <c r="I24" t="n">
-        <v>28.81</v>
+        <v>-715.65</v>
       </c>
       <c r="J24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K24" t="b">
         <v>0</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CHOLAFIN</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Cholamandalam Investment &amp; Finance Company Ltd</t>
+          <t xml:space="preserve">Cipla Ltd
+</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>-6.2</v>
+        <v>1.41</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Accrual Risk</t>
+          <t>High Quality</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>14.9</v>
+        <v>11.57</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1661,42 +1666,41 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>106.27</v>
+        <v>-22.43</v>
       </c>
       <c r="I25" t="n">
-        <v>-715.65</v>
+        <v>5.91</v>
       </c>
       <c r="J25" t="b">
+        <v>0</v>
+      </c>
+      <c r="K25" t="b">
         <v>1</v>
       </c>
-      <c r="K25" t="b">
-        <v>0</v>
-      </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cipla Ltd
-</t>
+          <t>Coal India Ltd</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1.41</v>
+        <v>1.02</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1704,24 +1708,24 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>11.57</v>
+        <v>3.15</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>-22.43</v>
+        <v>22.69</v>
       </c>
       <c r="I26" t="n">
-        <v>5.91</v>
+        <v>14.43</v>
       </c>
       <c r="J26" t="b">
         <v>0</v>
       </c>
       <c r="K26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -1732,21 +1736,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>DABUR</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Coal India Ltd</t>
+          <t>Dabur India Ltd</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1.02</v>
+        <v>1.08</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1754,7 +1758,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>3.15</v>
+        <v>7.83</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1762,10 +1766,10 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>22.69</v>
+        <v>-1.28</v>
       </c>
       <c r="I27" t="n">
-        <v>14.43</v>
+        <v>43.42</v>
       </c>
       <c r="J27" t="b">
         <v>0</v>
@@ -1782,29 +1786,29 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>DABUR</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Dabur India Ltd</t>
+          <t>Divis Laboratories Ltd</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1.08</v>
+        <v>0.93</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>7.83</v>
+        <v>3.43</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1812,10 +1816,10 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>-1.28</v>
+        <v>-3.27</v>
       </c>
       <c r="I28" t="n">
-        <v>43.42</v>
+        <v>44.89</v>
       </c>
       <c r="J28" t="b">
         <v>0</v>
@@ -1825,28 +1829,28 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>DLF</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Divis Laboratories Ltd</t>
+          <t>DLF Ltd</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.93</v>
+        <v>0.95</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1854,18 +1858,18 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>3.43</v>
+        <v>23.79</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="H29" t="n">
-        <v>-3.27</v>
+        <v>-38.07</v>
       </c>
       <c r="I29" t="n">
-        <v>44.89</v>
+        <v>47.55</v>
       </c>
       <c r="J29" t="b">
         <v>0</v>
@@ -1875,47 +1879,47 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>DLF</t>
+          <t>DMART</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>DLF Ltd</t>
+          <t>Avenue Supermarts Ltd</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.95</v>
+        <v>1.07</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
+          <t>High Quality</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>4.86</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="F30" t="n">
-        <v>23.79</v>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Capital Intensive</t>
-        </is>
-      </c>
       <c r="H30" t="n">
-        <v>-38.07</v>
+        <v>-46.44</v>
       </c>
       <c r="I30" t="n">
-        <v>47.55</v>
+        <v>6.77</v>
       </c>
       <c r="J30" t="b">
         <v>0</v>
@@ -1925,28 +1929,28 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>DMART</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Avenue Supermarts Ltd</t>
+          <t>Dr Reddys Laboratories Ltd</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1.07</v>
+        <v>1.34</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1954,18 +1958,18 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>4.86</v>
+        <v>14.4</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>-46.44</v>
+        <v>-32.75</v>
       </c>
       <c r="I31" t="n">
-        <v>6.77</v>
+        <v>6.42</v>
       </c>
       <c r="J31" t="b">
         <v>0</v>
@@ -1982,29 +1986,29 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Dr Reddys Laboratories Ltd</t>
+          <t>Eicher Motors Ltd</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1.34</v>
+        <v>1</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>14.4</v>
+        <v>17.14</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -2012,41 +2016,41 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>-32.75</v>
+        <v>47.9</v>
       </c>
       <c r="I32" t="n">
-        <v>6.42</v>
+        <v>20.56</v>
       </c>
       <c r="J32" t="b">
         <v>0</v>
       </c>
       <c r="K32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>GAIL</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Eicher Motors Ltd</t>
+          <t>GAIL (India) Ltd</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>0.99</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -2054,18 +2058,18 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>17.14</v>
+        <v>6.17</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>47.9</v>
+        <v>212.02</v>
       </c>
       <c r="I33" t="n">
-        <v>20.56</v>
+        <v>30.46</v>
       </c>
       <c r="J33" t="b">
         <v>0</v>
@@ -2082,79 +2086,79 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>GAIL</t>
+          <t>GODREJCP</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>GAIL (India) Ltd</t>
+          <t>Godrej Consumer Products Ltd</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.99</v>
+        <v>0.13</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Accrual Risk</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>6.17</v>
+        <v>24.37</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="H34" t="n">
-        <v>212.02</v>
+        <v>7.14</v>
       </c>
       <c r="I34" t="n">
-        <v>30.46</v>
+        <v>-46.16</v>
       </c>
       <c r="J34" t="b">
         <v>0</v>
       </c>
       <c r="K34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GODREJCP</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Godrej Consumer Products Ltd</t>
+          <t>Grasim Industries Ltd</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.13</v>
+        <v>0.61</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Accrual Risk</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>24.37</v>
+        <v>17.65</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2162,32 +2166,32 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>7.14</v>
+        <v>59.28</v>
       </c>
       <c r="I35" t="n">
-        <v>-46.16</v>
+        <v>-124.41</v>
       </c>
       <c r="J35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K35" t="b">
         <v>0</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>HAL</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Grasim Industries Ltd</t>
+          <t>Hindustan Aeronautics Ltd</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2196,15 +2200,15 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.61</v>
+        <v>1.96</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>High Quality</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>17.65</v>
+        <v>21.11</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2212,32 +2216,32 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>59.28</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="I36" t="n">
-        <v>-124.41</v>
+        <v>18.61</v>
       </c>
       <c r="J36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K36" t="b">
         <v>0</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>HAL</t>
+          <t>HAVELLS</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Hindustan Aeronautics Ltd</t>
+          <t>Havells India Ltd</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2246,7 +2250,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1.96</v>
+        <v>1.05</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -2254,7 +2258,7 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>21.11</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -2262,10 +2266,10 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>72.90000000000001</v>
+        <v>4.68</v>
       </c>
       <c r="I37" t="n">
-        <v>18.61</v>
+        <v>17.81</v>
       </c>
       <c r="J37" t="b">
         <v>0</v>
@@ -2282,21 +2286,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>HAVELLS</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Havells India Ltd</t>
+          <t>HCL Technologies Ltd</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1.05</v>
+        <v>1.37</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -2304,18 +2308,18 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>8.699999999999999</v>
+        <v>6.01</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>4.68</v>
+        <v>98.17</v>
       </c>
       <c r="I38" t="n">
-        <v>17.81</v>
+        <v>65.45999999999999</v>
       </c>
       <c r="J38" t="b">
         <v>0</v>
@@ -2332,29 +2336,29 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>HCL Technologies Ltd</t>
+          <t>HDFC Bank Ltd</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1.37</v>
+        <v>0.23</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Accrual Risk</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>6.01</v>
+        <v>5.85</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -2362,10 +2366,10 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>98.17</v>
+        <v>18.2</v>
       </c>
       <c r="I39" t="n">
-        <v>65.45999999999999</v>
+        <v>20.48</v>
       </c>
       <c r="J39" t="b">
         <v>0</v>
@@ -2375,19 +2379,19 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Liquidating Assets</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>HDFC Bank Ltd</t>
+          <t>HDFC Life Insurance Company Ltd</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2396,26 +2400,26 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.23</v>
+        <v>5.83</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Accrual Risk</t>
+          <t>High Quality</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>5.85</v>
+        <v>13.42</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>18.2</v>
+        <v>63.89</v>
       </c>
       <c r="I40" t="n">
-        <v>20.48</v>
+        <v>-2.87</v>
       </c>
       <c r="J40" t="b">
         <v>0</v>
@@ -2425,28 +2429,29 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Liquidating Assets</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>HEROMOTOCO</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>HDFC Life Insurance Company Ltd</t>
+          <t xml:space="preserve">Hero MotoCorp Ltd
+</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>5.83</v>
+        <v>1.21</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -2454,24 +2459,24 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>13.42</v>
+        <v>4.84</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="H41" t="n">
-        <v>63.89</v>
+        <v>3.48</v>
       </c>
       <c r="I41" t="n">
-        <v>-2.87</v>
+        <v>9.51</v>
       </c>
       <c r="J41" t="b">
         <v>0</v>
       </c>
       <c r="K41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -2482,22 +2487,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>HEROMOTOCO</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hero MotoCorp Ltd
-</t>
+          <t>Hindalco Industries Ltd</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>1.21</v>
+        <v>2.77</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -2505,7 +2509,7 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>4.84</v>
+        <v>6.61</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -2513,16 +2517,16 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>3.48</v>
+        <v>15.41</v>
       </c>
       <c r="I42" t="n">
-        <v>9.51</v>
+        <v>5.1</v>
       </c>
       <c r="J42" t="b">
         <v>0</v>
       </c>
       <c r="K42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
@@ -2533,21 +2537,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Hindalco Industries Ltd</t>
+          <t xml:space="preserve">Hindustan Unilever Ltd
+</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>2.77</v>
+        <v>1.16</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2555,18 +2560,18 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>6.61</v>
+        <v>8.6</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="H43" t="n">
-        <v>15.41</v>
+        <v>1.89</v>
       </c>
       <c r="I43" t="n">
-        <v>5.1</v>
+        <v>21.48</v>
       </c>
       <c r="J43" t="b">
         <v>0</v>
@@ -2583,22 +2588,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hindustan Unilever Ltd
-</t>
+          <t>ICICI Bank Ltd</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>1.16</v>
+        <v>3.87</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -2606,7 +2610,7 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>8.6</v>
+        <v>90.73999999999999</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -2614,10 +2618,10 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>1.89</v>
+        <v>-23.93</v>
       </c>
       <c r="I44" t="n">
-        <v>21.48</v>
+        <v>12.6</v>
       </c>
       <c r="J44" t="b">
         <v>0</v>
@@ -2627,19 +2631,19 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>ICICIGI</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ICICI Bank Ltd</t>
+          <t>ICICI Lombard General Insurance Company Ltd</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2648,7 +2652,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>3.87</v>
+        <v>1.46</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2656,7 +2660,7 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>90.73999999999999</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -2664,32 +2668,32 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>-23.93</v>
+        <v>75.7</v>
       </c>
       <c r="I45" t="n">
-        <v>12.6</v>
+        <v>2.71</v>
       </c>
       <c r="J45" t="b">
         <v>0</v>
       </c>
       <c r="K45" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ICICIGI</t>
+          <t>ICICIPRULI</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ICICI Lombard General Insurance Company Ltd</t>
+          <t>ICICI Prudential Life Insurance Company Ltd</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2698,7 +2702,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>1.46</v>
+        <v>1.93</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -2706,7 +2710,7 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>9.380000000000001</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -2714,10 +2718,10 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>75.7</v>
+        <v>-53.26</v>
       </c>
       <c r="I46" t="n">
-        <v>2.71</v>
+        <v>0.11</v>
       </c>
       <c r="J46" t="b">
         <v>0</v>
@@ -2727,36 +2731,36 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Other</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ICICIPRULI</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ICICI Prudential Life Insurance Company Ltd</t>
+          <t>Interglobe Aviation Ltd</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1.93</v>
+        <v>-14.34</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Accrual Risk</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>8.220000000000001</v>
+        <v>17.07</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -2764,60 +2768,60 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>-53.26</v>
+        <v>41.21</v>
       </c>
       <c r="I47" t="n">
-        <v>0.11</v>
+        <v>17.93</v>
       </c>
       <c r="J47" t="b">
         <v>0</v>
       </c>
       <c r="K47" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>INDUSINDBK</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Interglobe Aviation Ltd</t>
+          <t>IndusInd Bank Ltd</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>-14.34</v>
+        <v>2.61</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Accrual Risk</t>
+          <t>High Quality</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>17.07</v>
+        <v>1.37</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Asset Light</t>
         </is>
       </c>
       <c r="H48" t="n">
-        <v>41.21</v>
+        <v>10.98</v>
       </c>
       <c r="I48" t="n">
-        <v>17.93</v>
+        <v>-99.04000000000001</v>
       </c>
       <c r="J48" t="b">
         <v>0</v>
@@ -2827,28 +2831,28 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
+          <t>Pre-Revenue</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>INDUSINDBK</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>IndusInd Bank Ltd</t>
+          <t>Infosys Ltd</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>2.61</v>
+        <v>1.04</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -2856,18 +2860,18 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>1.37</v>
+        <v>3.31</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Asset Light</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="H49" t="n">
-        <v>10.98</v>
+        <v>4.81</v>
       </c>
       <c r="I49" t="n">
-        <v>-99.04000000000001</v>
+        <v>55.23</v>
       </c>
       <c r="J49" t="b">
         <v>0</v>
@@ -2877,36 +2881,37 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Pre-Revenue</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>IOC</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Infosys Ltd</t>
+          <t xml:space="preserve">Indian Oil Corporation
+</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1.04</v>
+        <v>0.73</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>3.31</v>
+        <v>4.05</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2914,10 +2919,10 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>4.81</v>
+        <v>15.91</v>
       </c>
       <c r="I50" t="n">
-        <v>55.23</v>
+        <v>52.4</v>
       </c>
       <c r="J50" t="b">
         <v>0</v>
@@ -2927,29 +2932,28 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>IOC</t>
+          <t>IRCTC</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Indian Oil Corporation
-</t>
+          <t>Indian Railway Catering &amp; Tourism Corporation Ltd</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.73</v>
+        <v>0.9</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -2957,7 +2961,7 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>4.05</v>
+        <v>5.04</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2965,16 +2969,16 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>15.91</v>
+        <v>12.46</v>
       </c>
       <c r="I51" t="n">
-        <v>52.4</v>
+        <v>45.5</v>
       </c>
       <c r="J51" t="b">
         <v>0</v>
       </c>
       <c r="K51" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -2985,40 +2989,40 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>IRCTC</t>
+          <t>IRFC</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Indian Railway Catering &amp; Tourism Corporation Ltd</t>
+          <t>Indian Railway Finance Corporation Ltd</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.9</v>
+        <v>-10.8</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Accrual Risk</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>5.04</v>
+        <v>0.03</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Asset Light</t>
         </is>
       </c>
       <c r="H52" t="n">
-        <v>12.46</v>
+        <v>-40.41</v>
       </c>
       <c r="I52" t="n">
-        <v>45.5</v>
+        <v>29.82</v>
       </c>
       <c r="J52" t="b">
         <v>0</v>
@@ -3035,29 +3039,30 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>IRFC</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Indian Railway Finance Corporation Ltd</t>
+          <t xml:space="preserve">ITC Ltd
+</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>-10.8</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Accrual Risk</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>0.03</v>
+        <v>2.21</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -3065,61 +3070,60 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>-40.41</v>
+        <v>21.8</v>
       </c>
       <c r="I53" t="n">
-        <v>29.82</v>
+        <v>71.44</v>
       </c>
       <c r="J53" t="b">
         <v>0</v>
       </c>
       <c r="K53" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
+          <t>Liquidating Assets</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>JINDALSTEL</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">ITC Ltd
-</t>
+          <t>Jindal Steel &amp; Power Ltd</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.9399999999999999</v>
+        <v>-2.8</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Accrual Risk</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>2.21</v>
+        <v>16.57</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Asset Light</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="H54" t="n">
-        <v>21.8</v>
+        <v>-24.89</v>
       </c>
       <c r="I54" t="n">
-        <v>71.44</v>
+        <v>-22.9</v>
       </c>
       <c r="J54" t="b">
         <v>0</v>
@@ -3129,47 +3133,45 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>Liquidating Assets</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>JINDALSTEL</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Jindal Steel &amp; Power Ltd</t>
+          <t>Jio Financial Services Ltd</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>-2.8</v>
+        <v>32.93</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Accrual Risk</t>
+          <t>High Quality</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>16.57</v>
+        <v>77.68000000000001</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H55" t="n">
-        <v>-24.89</v>
-      </c>
+      <c r="H55" t="inlineStr"/>
       <c r="I55" t="n">
-        <v>-22.9</v>
+        <v>48.94</v>
       </c>
       <c r="J55" t="b">
         <v>0</v>
@@ -3179,28 +3181,28 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Other</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>JSWENERGY</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Jio Financial Services Ltd</t>
+          <t>JSW Energy Ltd</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>32.93</v>
+        <v>2.63</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -3208,16 +3210,18 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>77.68000000000001</v>
+        <v>71.37</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
           <t>Capital Intensive</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
+      <c r="H56" t="n">
+        <v>-4.73</v>
+      </c>
       <c r="I56" t="n">
-        <v>48.94</v>
+        <v>-36.47</v>
       </c>
       <c r="J56" t="b">
         <v>0</v>
@@ -3227,28 +3231,28 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>JSWENERGY</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>JSW Energy Ltd</t>
+          <t>JSW Steel Ltd</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>2.63</v>
+        <v>2.78</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -3256,7 +3260,7 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>71.37</v>
+        <v>8.27</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -3264,10 +3268,10 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>-4.73</v>
+        <v>-23.02</v>
       </c>
       <c r="I57" t="n">
-        <v>-36.47</v>
+        <v>-8.48</v>
       </c>
       <c r="J57" t="b">
         <v>0</v>
@@ -3277,28 +3281,29 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>JSW Steel Ltd</t>
+          <t xml:space="preserve">Kotak Mahindra Bank Ltd
+</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>2.78</v>
+        <v>1.48</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -3306,7 +3311,7 @@
         </is>
       </c>
       <c r="F58" t="n">
-        <v>8.27</v>
+        <v>15.86</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -3314,10 +3319,10 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>-23.02</v>
+        <v>-32.99</v>
       </c>
       <c r="I58" t="n">
-        <v>-8.48</v>
+        <v>14.38</v>
       </c>
       <c r="J58" t="b">
         <v>0</v>
@@ -3327,20 +3332,19 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>LICI</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kotak Mahindra Bank Ltd
-</t>
+          <t>Life Insurance Corporation of India</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3349,7 +3353,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1.48</v>
+        <v>9.68</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -3357,18 +3361,18 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>15.86</v>
+        <v>2.99</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Asset Light</t>
         </is>
       </c>
       <c r="H59" t="n">
-        <v>-32.99</v>
+        <v>-50.27</v>
       </c>
       <c r="I59" t="n">
-        <v>14.38</v>
+        <v>2.6</v>
       </c>
       <c r="J59" t="b">
         <v>0</v>
@@ -3378,28 +3382,28 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>LICI</t>
+          <t>LODHA</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Life Insurance Corporation of India</t>
+          <t>Macrotech Developers Ltd</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>9.68</v>
+        <v>13.31</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -3407,18 +3411,18 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>2.99</v>
+        <v>28.57</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Asset Light</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="H60" t="n">
-        <v>-50.27</v>
+        <v>-42.41</v>
       </c>
       <c r="I60" t="n">
-        <v>2.6</v>
+        <v>-16.32</v>
       </c>
       <c r="J60" t="b">
         <v>0</v>
@@ -3428,28 +3432,28 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>LODHA</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Macrotech Developers Ltd</t>
+          <t>Larsen &amp; Toubro Ltd</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>13.31</v>
+        <v>1.45</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -3457,18 +3461,18 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>28.57</v>
+        <v>0.99</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Asset Light</t>
         </is>
       </c>
       <c r="H61" t="n">
-        <v>-42.41</v>
+        <v>85.84</v>
       </c>
       <c r="I61" t="n">
-        <v>-16.32</v>
+        <v>68.45999999999999</v>
       </c>
       <c r="J61" t="b">
         <v>0</v>
@@ -3478,28 +3482,28 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Liquidating Assets</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>LTIM</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Larsen &amp; Toubro Ltd</t>
+          <t>LTIMindtree Ltd</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>1.45</v>
+        <v>1.02</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -3507,18 +3511,18 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>0.99</v>
+        <v>11.03</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Asset Light</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="H62" t="n">
-        <v>85.84</v>
+        <v>15.02</v>
       </c>
       <c r="I62" t="n">
-        <v>68.45999999999999</v>
+        <v>27.43</v>
       </c>
       <c r="J62" t="b">
         <v>0</v>
@@ -3528,28 +3532,29 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>Liquidating Assets</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>LTIM</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>LTIMindtree Ltd</t>
+          <t xml:space="preserve">Mahindra &amp; Mahindra Ltd
+</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1.02</v>
+        <v>3.32</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -3557,41 +3562,40 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>11.03</v>
+        <v>4.04</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="H63" t="n">
-        <v>15.02</v>
+        <v>7.8</v>
       </c>
       <c r="I63" t="n">
-        <v>27.43</v>
+        <v>-45.18</v>
       </c>
       <c r="J63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K63" t="b">
         <v>0</v>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mahindra &amp; Mahindra Ltd
-</t>
+          <t>Maruti Suzuki India Ltd</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3600,7 +3604,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>3.32</v>
+        <v>1.13</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -3608,40 +3612,40 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>4.04</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="H64" t="n">
-        <v>7.8</v>
+        <v>13.84</v>
       </c>
       <c r="I64" t="n">
-        <v>-45.18</v>
+        <v>26.5</v>
       </c>
       <c r="J64" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K64" t="b">
         <v>0</v>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>MOTHERSON</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Maruti Suzuki India Ltd</t>
+          <t>Samvardhana Motherson International Ltd</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3650,7 +3654,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>1.13</v>
+        <v>3.1</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -3658,18 +3662,18 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>8.359999999999999</v>
+        <v>6.73</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="H65" t="n">
-        <v>13.84</v>
+        <v>-31.21</v>
       </c>
       <c r="I65" t="n">
-        <v>26.5</v>
+        <v>9.92</v>
       </c>
       <c r="J65" t="b">
         <v>0</v>
@@ -3679,47 +3683,47 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>MOTHERSON</t>
+          <t>NAUKRI</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Samvardhana Motherson International Ltd</t>
+          <t>Info Edge (India) Ltd</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>3.1</v>
+        <v>-1.46</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Accrual Risk</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>6.73</v>
+        <v>33.6</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="H66" t="n">
-        <v>-31.21</v>
+        <v>-23.89</v>
       </c>
       <c r="I66" t="n">
-        <v>9.92</v>
+        <v>-21.1</v>
       </c>
       <c r="J66" t="b">
         <v>0</v>
@@ -3736,40 +3740,40 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>NAUKRI</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Info Edge (India) Ltd</t>
+          <t>Nestle India Ltd</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>-1.46</v>
+        <v>1.11</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Accrual Risk</t>
+          <t>High Quality</t>
         </is>
       </c>
       <c r="F67" t="n">
-        <v>33.6</v>
+        <v>5.07</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="H67" t="n">
-        <v>-23.89</v>
+        <v>8.33</v>
       </c>
       <c r="I67" t="n">
-        <v>-21.1</v>
+        <v>50.54</v>
       </c>
       <c r="J67" t="b">
         <v>0</v>
@@ -3779,28 +3783,29 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>NHPC</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Nestle India Ltd</t>
+          <t xml:space="preserve">NHPC Ltd
+</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>1.11</v>
+        <v>1.27</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -3808,18 +3813,18 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>5.07</v>
+        <v>61.96</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="H68" t="n">
-        <v>8.33</v>
+        <v>256.58</v>
       </c>
       <c r="I68" t="n">
-        <v>50.54</v>
+        <v>20.18</v>
       </c>
       <c r="J68" t="b">
         <v>0</v>
@@ -3836,13 +3841,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>NHPC</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">NHPC Ltd
-</t>
+          <t>NTPC Ltd</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3851,7 +3855,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>1.27</v>
+        <v>2.26</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -3859,7 +3863,7 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>61.96</v>
+        <v>18.01</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -3867,10 +3871,10 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>256.58</v>
+        <v>10.79</v>
       </c>
       <c r="I69" t="n">
-        <v>20.18</v>
+        <v>16.8</v>
       </c>
       <c r="J69" t="b">
         <v>0</v>
@@ -3887,12 +3891,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>NTPC Ltd</t>
+          <t>Oil &amp; Natural Gas Corpn Ltd</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3901,7 +3905,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>2.26</v>
+        <v>2.86</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -3909,7 +3913,7 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>18.01</v>
+        <v>9.67</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -3917,10 +3921,10 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>10.79</v>
+        <v>24.63</v>
       </c>
       <c r="I70" t="n">
-        <v>16.8</v>
+        <v>40.9</v>
       </c>
       <c r="J70" t="b">
         <v>0</v>
@@ -3937,320 +3941,320 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>PFC</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Oil &amp; Natural Gas Corpn Ltd</t>
+          <t>Power Finance Corporation Ltd</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>2.86</v>
+        <v>-3.03</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Accrual Risk</t>
         </is>
       </c>
       <c r="F71" t="n">
-        <v>9.67</v>
+        <v>3.73</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="H71" t="n">
-        <v>24.63</v>
+        <v>24.44</v>
       </c>
       <c r="I71" t="n">
-        <v>40.9</v>
+        <v>-301.52</v>
       </c>
       <c r="J71" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K71" t="b">
         <v>0</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>PFC</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Power Finance Corporation Ltd</t>
+          <t>Pidilite Industries Ltd</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>-3.03</v>
+        <v>1.19</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Accrual Risk</t>
+          <t>High Quality</t>
         </is>
       </c>
       <c r="F72" t="n">
-        <v>3.73</v>
+        <v>14.29</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="H72" t="n">
-        <v>24.44</v>
+        <v>-8.84</v>
       </c>
       <c r="I72" t="n">
-        <v>-301.52</v>
+        <v>35.27</v>
       </c>
       <c r="J72" t="b">
+        <v>0</v>
+      </c>
+      <c r="K72" t="b">
         <v>1</v>
       </c>
-      <c r="K72" t="b">
-        <v>0</v>
-      </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>PNB</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Pidilite Industries Ltd</t>
+          <t>Punjab National Bank</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>1.19</v>
+        <v>-1.22</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Accrual Risk</t>
         </is>
       </c>
       <c r="F73" t="n">
-        <v>14.29</v>
+        <v>1.38</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Asset Light</t>
         </is>
       </c>
       <c r="H73" t="n">
-        <v>-8.84</v>
-      </c>
-      <c r="I73" t="n">
-        <v>35.27</v>
-      </c>
+        <v>22.37</v>
+      </c>
+      <c r="I73" t="inlineStr"/>
       <c r="J73" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K73" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Punjab National Bank</t>
+          <t>Power Grid Corporation of India Ltd</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>-1.22</v>
+        <v>2.36</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Accrual Risk</t>
+          <t>High Quality</t>
         </is>
       </c>
       <c r="F74" t="n">
-        <v>1.38</v>
+        <v>28.61</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Asset Light</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="H74" t="n">
-        <v>22.37</v>
-      </c>
-      <c r="I74" t="inlineStr"/>
+        <v>4.85</v>
+      </c>
+      <c r="I74" t="n">
+        <v>60.7</v>
+      </c>
       <c r="J74" t="b">
+        <v>0</v>
+      </c>
+      <c r="K74" t="b">
         <v>1</v>
       </c>
-      <c r="K74" t="b">
-        <v>0</v>
-      </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>RECLTD</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Power Grid Corporation of India Ltd</t>
+          <t>REC Ltd</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>2.36</v>
+        <v>-3.86</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Accrual Risk</t>
         </is>
       </c>
       <c r="F75" t="n">
-        <v>28.61</v>
+        <v>3.85</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="H75" t="n">
-        <v>4.85</v>
+        <v>16.27</v>
       </c>
       <c r="I75" t="n">
-        <v>60.7</v>
+        <v>-124.37</v>
       </c>
       <c r="J75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K75" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>RECLTD</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>REC Ltd</t>
+          <t xml:space="preserve">Reliance Industries Ltd
+</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>-3.86</v>
+        <v>1.61</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Accrual Risk</t>
+          <t>High Quality</t>
         </is>
       </c>
       <c r="F76" t="n">
-        <v>3.85</v>
+        <v>12.63</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="H76" t="n">
-        <v>16.27</v>
+        <v>19.22</v>
       </c>
       <c r="I76" t="n">
-        <v>-124.37</v>
+        <v>27.82</v>
       </c>
       <c r="J76" t="b">
+        <v>0</v>
+      </c>
+      <c r="K76" t="b">
         <v>1</v>
       </c>
-      <c r="K76" t="b">
-        <v>0</v>
-      </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reliance Industries Ltd
-</t>
+          <t>SBI Life Insurance Company Ltd</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1.61</v>
+        <v>15.3</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -4258,7 +4262,7 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>12.63</v>
+        <v>23.65</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -4266,16 +4270,16 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>19.22</v>
+        <v>-2.4</v>
       </c>
       <c r="I77" t="n">
-        <v>27.82</v>
+        <v>-853.25</v>
       </c>
       <c r="J77" t="b">
         <v>0</v>
       </c>
       <c r="K77" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L77" t="inlineStr">
         <is>
@@ -4286,12 +4290,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SBI Life Insurance Company Ltd</t>
+          <t>State Bank of India</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -4300,7 +4304,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>15.3</v>
+        <v>1.05</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -4308,18 +4312,18 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>23.65</v>
+        <v>0.79</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Asset Light</t>
         </is>
       </c>
       <c r="H78" t="n">
-        <v>-2.4</v>
+        <v>-6.12</v>
       </c>
       <c r="I78" t="n">
-        <v>-853.25</v>
+        <v>-30.11</v>
       </c>
       <c r="J78" t="b">
         <v>0</v>
@@ -4336,21 +4340,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>SHREECEM</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>State Bank of India</t>
+          <t>Shree Cement Ltd</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>1.05</v>
+        <v>1.9</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -4358,18 +4362,18 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>0.79</v>
+        <v>6.91</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Asset Light</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="H79" t="n">
-        <v>-6.12</v>
+        <v>4.51</v>
       </c>
       <c r="I79" t="n">
-        <v>-30.11</v>
+        <v>42.7</v>
       </c>
       <c r="J79" t="b">
         <v>0</v>
@@ -4386,80 +4390,80 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>SHREECEM</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Shree Cement Ltd</t>
+          <t xml:space="preserve">Shriram Finance Ltd
+</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>1.9</v>
+        <v>-2.61</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Accrual Risk</t>
         </is>
       </c>
       <c r="F80" t="n">
-        <v>6.91</v>
+        <v>0.71</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Asset Light</t>
         </is>
       </c>
       <c r="H80" t="n">
-        <v>4.51</v>
+        <v>87.84</v>
       </c>
       <c r="I80" t="n">
-        <v>42.7</v>
+        <v>-298</v>
       </c>
       <c r="J80" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K80" t="b">
         <v>0</v>
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>SIEMENS</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shriram Finance Ltd
-</t>
+          <t>Siemens Ltd</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>-2.61</v>
+        <v>0.84</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Accrual Risk</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="F81" t="n">
-        <v>0.71</v>
+        <v>2.26</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -4467,49 +4471,49 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>87.84</v>
+        <v>-7.44</v>
       </c>
       <c r="I81" t="n">
-        <v>-298</v>
+        <v>37.63</v>
       </c>
       <c r="J81" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K81" t="b">
         <v>0</v>
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SIEMENS</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Siemens Ltd</t>
+          <t>Sun Pharmaceuticals Industries Ltd</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0.84</v>
+        <v>1.76</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>High Quality</t>
         </is>
       </c>
       <c r="F82" t="n">
-        <v>2.26</v>
+        <v>1.57</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -4517,41 +4521,41 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>-7.44</v>
+        <v>27.3</v>
       </c>
       <c r="I82" t="n">
-        <v>37.63</v>
+        <v>87.36</v>
       </c>
       <c r="J82" t="b">
         <v>0</v>
       </c>
       <c r="K82" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Sun Pharmaceuticals Industries Ltd</t>
+          <t>Tata Consumer Products Ltd</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>1.76</v>
+        <v>1.67</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -4559,49 +4563,49 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>1.57</v>
+        <v>12.57</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Asset Light</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="H83" t="n">
-        <v>27.3</v>
+        <v>-51.24</v>
       </c>
       <c r="I83" t="n">
-        <v>87.36</v>
+        <v>1.14</v>
       </c>
       <c r="J83" t="b">
         <v>0</v>
       </c>
       <c r="K83" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>TATAMOTORS</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Tata Consumer Products Ltd</t>
+          <t>Tata Motors Ltd</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>1.67</v>
+        <v>1.93</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -4609,49 +4613,50 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>12.57</v>
+        <v>5.2</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="H84" t="n">
-        <v>-51.24</v>
+        <v>62.44</v>
       </c>
       <c r="I84" t="n">
-        <v>1.14</v>
+        <v>75.81</v>
       </c>
       <c r="J84" t="b">
         <v>0</v>
       </c>
       <c r="K84" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>TATAMOTORS</t>
+          <t>TATAPOWER</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Tata Motors Ltd</t>
+          <t xml:space="preserve">Tata Power Company Ltd
+</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>1.93</v>
+        <v>3.87</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -4659,24 +4664,24 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>5.2</v>
+        <v>14.69</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Capital Intensive</t>
         </is>
       </c>
       <c r="H85" t="n">
-        <v>62.44</v>
+        <v>-15.14</v>
       </c>
       <c r="I85" t="n">
-        <v>75.81</v>
+        <v>33.25</v>
       </c>
       <c r="J85" t="b">
         <v>0</v>
       </c>
       <c r="K85" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L85" t="inlineStr">
         <is>
@@ -4687,22 +4692,22 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>TATAPOWER</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tata Power Company Ltd
+          <t xml:space="preserve">Tata Steel Ltd
 </t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>3.87</v>
+        <v>4.44</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -4710,18 +4715,18 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>14.69</v>
+        <v>6.22</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="H86" t="n">
-        <v>-15.14</v>
+        <v>-0.45</v>
       </c>
       <c r="I86" t="n">
-        <v>33.25</v>
+        <v>27.18</v>
       </c>
       <c r="J86" t="b">
         <v>0</v>
@@ -4738,22 +4743,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tata Steel Ltd
-</t>
+          <t>Tata Consultancy Services Ltd</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>4.44</v>
+        <v>1.04</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -4761,18 +4765,18 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>6.22</v>
+        <v>2.53</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Asset Light</t>
         </is>
       </c>
       <c r="H87" t="n">
-        <v>-0.45</v>
+        <v>5.1</v>
       </c>
       <c r="I87" t="n">
-        <v>27.18</v>
+        <v>78.43000000000001</v>
       </c>
       <c r="J87" t="b">
         <v>0</v>
@@ -4782,19 +4786,19 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Liquidating Assets</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Tata Consultancy Services Ltd</t>
+          <t>Tech Mahindra Ltd</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -4803,7 +4807,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>1.04</v>
+        <v>1.54</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -4819,49 +4823,50 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>5.1</v>
+        <v>-1.8</v>
       </c>
       <c r="I88" t="n">
-        <v>78.43000000000001</v>
+        <v>112.25</v>
       </c>
       <c r="J88" t="b">
         <v>0</v>
       </c>
       <c r="K88" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>Liquidating Assets</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Tech Mahindra Ltd</t>
+          <t xml:space="preserve">Titan Company Ltd
+</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>1.54</v>
+        <v>0.92</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="F89" t="n">
-        <v>2.53</v>
+        <v>0.37</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -4869,50 +4874,49 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>-1.8</v>
+        <v>91.06999999999999</v>
       </c>
       <c r="I89" t="n">
-        <v>112.25</v>
+        <v>28.46</v>
       </c>
       <c r="J89" t="b">
         <v>0</v>
       </c>
       <c r="K89" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>TORNTPHARM</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Titan Company Ltd
-</t>
+          <t>Torrent Pharmaceuticals Ltd</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>0.92</v>
+        <v>1.83</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>High Quality</t>
         </is>
       </c>
       <c r="F90" t="n">
-        <v>0.37</v>
+        <v>1.49</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -4920,41 +4924,41 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>91.06999999999999</v>
+        <v>17.64</v>
       </c>
       <c r="I90" t="n">
-        <v>28.46</v>
+        <v>92.22</v>
       </c>
       <c r="J90" t="b">
         <v>0</v>
       </c>
       <c r="K90" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>TORNTPHARM</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Torrent Pharmaceuticals Ltd</t>
+          <t>Trent Ltd</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>1.83</v>
+        <v>1.18</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -4962,24 +4966,24 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>1.49</v>
+        <v>4.11</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Asset Light</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="H91" t="n">
-        <v>17.64</v>
+        <v>17.05</v>
       </c>
       <c r="I91" t="n">
-        <v>92.22</v>
+        <v>42.67</v>
       </c>
       <c r="J91" t="b">
         <v>0</v>
       </c>
       <c r="K91" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -4990,12 +4994,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>TVSMOTOR</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Trent Ltd</t>
+          <t>TVS Motor Company Ltd</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -5004,84 +5008,34 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>1.18</v>
+        <v>-0.75</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Accrual Risk</t>
         </is>
       </c>
       <c r="F92" t="n">
-        <v>4.11</v>
+        <v>2.56</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Asset Light</t>
         </is>
       </c>
       <c r="H92" t="n">
-        <v>17.05</v>
+        <v>33.16</v>
       </c>
       <c r="I92" t="n">
-        <v>42.67</v>
+        <v>-40.98</v>
       </c>
       <c r="J92" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K92" t="b">
         <v>0</v>
       </c>
       <c r="L92" t="inlineStr">
-        <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>TVSMOTOR</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>TVS Motor Company Ltd</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
-      <c r="D93" t="n">
-        <v>-0.75</v>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>Accrual Risk</t>
-        </is>
-      </c>
-      <c r="F93" t="n">
-        <v>2.56</v>
-      </c>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>Asset Light</t>
-        </is>
-      </c>
-      <c r="H93" t="n">
-        <v>33.16</v>
-      </c>
-      <c r="I93" t="n">
-        <v>-40.98</v>
-      </c>
-      <c r="J93" t="b">
-        <v>1</v>
-      </c>
-      <c r="K93" t="b">
-        <v>0</v>
-      </c>
-      <c r="L93" t="inlineStr">
         <is>
           <t>Growth Funded by Debt</t>
         </is>

</xml_diff>